<commit_message>
fix(finance): audit GC02 economic truth
</commit_message>
<xml_diff>
--- a/packages/testing-fixtures/assets/camil-management/01_Orcamento_2026_2027.xlsx
+++ b/packages/testing-fixtures/assets/camil-management/01_Orcamento_2026_2027.xlsx
@@ -398,6 +398,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F14"/>
+  <cols>
+    <col min="1" max="1" width="46.83203125" customWidth="1"/>
+    <col min="2" max="2" width="22.83203125" customWidth="1"/>
+    <col min="3" max="3" width="22.83203125" customWidth="1"/>
+    <col min="4" max="4" width="22.83203125" customWidth="1"/>
+    <col min="5" max="5" width="22.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>

<commit_message>
fix(finance): audit GC02 economic truth (#516)
</commit_message>
<xml_diff>
--- a/packages/testing-fixtures/assets/camil-management/01_Orcamento_2026_2027.xlsx
+++ b/packages/testing-fixtures/assets/camil-management/01_Orcamento_2026_2027.xlsx
@@ -398,6 +398,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:F14"/>
+  <cols>
+    <col min="1" max="1" width="46.83203125" customWidth="1"/>
+    <col min="2" max="2" width="22.83203125" customWidth="1"/>
+    <col min="3" max="3" width="22.83203125" customWidth="1"/>
+    <col min="4" max="4" width="22.83203125" customWidth="1"/>
+    <col min="5" max="5" width="22.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">

</xml_diff>